<commit_message>
Enhance test suite configuration in testng.xml for improved parallel execution; add new Mixed Advanced Filters load test. Introduce detailed Allure report HTML file for better test reporting. Update basePage for cleaner WebDriver setup and add new utility classes for language and professional details filters, including Excel management. Refactor existing filter utilities to remove sample data in templates.
</commit_message>
<xml_diff>
--- a/src/test/resources/advanced_filters_excel_sheets/filters_ctc.xlsx
+++ b/src/test/resources/advanced_filters_excel_sheets/filters_ctc.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\workspace-spring-tools-for-eclipse-4.31.0.RELEASE\SSWebsite\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Downloads\Eticaa Project Automation\Eticaa-Automation\src\test\resources\advanced_filters_excel_sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97FDE1E2-1A06-4907-9AF7-62A6AE39742F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5399D50C-0655-4345-9FE6-FE05AB19F716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="ExperienceRanges" sheetId="1" r:id="rId1"/>
+    <sheet name="CurrrentCTCFilters" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -381,9 +381,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -391,7 +391,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -399,7 +399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -407,7 +407,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -415,7 +415,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>5</v>
       </c>
@@ -423,7 +423,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>8</v>
       </c>
@@ -431,7 +431,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -439,7 +439,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -447,7 +447,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>0</v>
       </c>
@@ -455,7 +455,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -463,7 +463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2</v>
       </c>
@@ -471,7 +471,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>4</v>
       </c>
@@ -479,7 +479,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>6</v>
       </c>
@@ -487,7 +487,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>10</v>
       </c>
@@ -495,7 +495,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>15</v>
       </c>
@@ -503,7 +503,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>20</v>
       </c>
@@ -511,7 +511,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>-5</v>
       </c>
@@ -519,7 +519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>0</v>
       </c>
@@ -527,7 +527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1</v>
       </c>
@@ -535,7 +535,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>2</v>
       </c>
@@ -543,7 +543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>50</v>
       </c>

</xml_diff>